<commit_message>
Correr las 3 corridas reales contra la API de Anthropic y corregir bug de promedio de ingresos
- agente/correr_corridas_reales.py: driver para correr el agente real contra corridas/*/entrada.md
- agente/tools.py: evaluar_legajo ahora recibe la lista cruda de ingresos y promedia internamente (antes el LLM promediaba mal en un caso real)
- prompts/, agente/legajo_agent.py: reglas explicitas sobre no promediar a mano y usar 'Credito Aprobado' (no 'Total Credito con fee') para LTV
- corridas/, output/legajos_maestro.xlsx: resultado y costo reales de response.usage
- DECISIONES.md, ANALISIS_ECONOMICO.md, GOBIERNO_Y_RIESGO.md: iteraciones 8 y 9 documentando el hallazgo y la correccion
</commit_message>
<xml_diff>
--- a/output/legajos_maestro.xlsx
+++ b/output/legajos_maestro.xlsx
@@ -553,7 +553,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Juan Perez</t>
+          <t>Perez</t>
         </is>
       </c>
       <c r="D2" s="2" t="n">
@@ -614,12 +614,12 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Mar del Plata</t>
+          <t>MAR DEL PLATA</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Pablo Gonzalez</t>
+          <t>Gonzalez</t>
         </is>
       </c>
       <c r="D3" s="2" t="n">
@@ -680,7 +680,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Córdoba</t>
+          <t>CORDOBA</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">

</xml_diff>

<commit_message>
Detectar ingresos atipicos y priorizar comprobantes reales sobre el Resumen Carpeta
- El usuario noto que el ingreso de agosto de Lopez no coincide con los comprobantes reales de la carpeta Ingresos de Drive
- Se verifico contra los 3 legajos: Lopez tiene 2 meses mal cargados (julio y agosto), Perez y Gonzalez coinciden
- agente/tools.py: promediar_ingresos ahora detecta meses atipicos (>3x la mediana) y los reporta en 'advertencias', independiente del resultado de los controles
- prompts/, legajo_agent.py: regla explicita de priorizar comprobantes reales sobre el resumen cuando hay discrepancia
- corridas/*/entrada.md: agregada verificacion cruzada contra comprobantes reales para los 3 legajos
- Re-corridas reales contra la API con los datos corregidos (Lopez: Control 1 pasa de 43.2% a 41.5%, sigue rechazado, ahora con advertencia de ingreso atipico)
- DECISIONES.md Iteracion 10, GOBIERNO_Y_RIESGO.md y ANALISIS_ECONOMICO.md actualizados con el hallazgo y el costo real final
</commit_message>
<xml_diff>
--- a/output/legajos_maestro.xlsx
+++ b/output/legajos_maestro.xlsx
@@ -557,13 +557,13 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>2707521.33</v>
+        <v>2722000</v>
       </c>
       <c r="E2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>2707521.33</v>
+        <v>2722000</v>
       </c>
       <c r="G2" s="2" t="n">
         <v>488.04</v>
@@ -576,7 +576,7 @@
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>27.3%</t>
+          <t>27.2%</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -689,13 +689,13 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>1702509.5</v>
+        <v>1771354.5</v>
       </c>
       <c r="E4" t="n">
         <v>0</v>
       </c>
       <c r="F4" t="n">
-        <v>1702509.5</v>
+        <v>1771354.5</v>
       </c>
       <c r="G4" t="n">
         <v>523.47</v>
@@ -708,7 +708,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>43.2%</t>
+          <t>41.5%</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -734,7 +734,7 @@
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>credito no aprobado — Relación cuota/ingreso de 43.2% supera el límite de 40%; LTV de 40.5% supera el límite de 35%</t>
+          <t>credito no aprobado — Relación cuota/ingreso de 41.5% supera el límite de 40%; LTV de 40.5% supera el límite de 35%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Evidencia real: 3 legajos de negocio + caso de prueba incompleto, con corridas versionadas
- Re-corridas de Perez, Gonzalez y Lopez contra la API real con el nuevo esquema (acepta null, datos_faltantes)
- Nueva corrida real: corrida_04_incompleto (Martinez, sin valor de propiedad) -> resultado_final: no evaluable, datos_faltantes: [valor_propiedad_usd], sin inventar ningun numero
- Cada corrida queda archivada en corridas/<caso>/runs/<timestamp>/ sin sobrescribir corridas anteriores
- output/legajos_maestro.xlsx regenerado (solo 3 legajos de negocio, el caso de prueba no entra)
- DECISIONES.md Iteracion 11, ANALISIS_ECONOMICO.md y GOBIERNO_Y_RIESGO.md actualizados con el costo real y el cierre de los 3 hallazgos del agente evaluador del grupo (96/100)
</commit_message>
<xml_diff>
--- a/output/legajos_maestro.xlsx
+++ b/output/legajos_maestro.xlsx
@@ -559,9 +559,7 @@
       <c r="D2" s="2" t="n">
         <v>2722000</v>
       </c>
-      <c r="E2" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="E2" s="2" t="n"/>
       <c r="F2" s="2" t="n">
         <v>2722000</v>
       </c>
@@ -625,9 +623,7 @@
       <c r="D3" s="2" t="n">
         <v>2709944.17</v>
       </c>
-      <c r="E3" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="E3" s="2" t="n"/>
       <c r="F3" s="2" t="n">
         <v>2709944.17</v>
       </c>
@@ -690,9 +686,6 @@
       </c>
       <c r="D4" t="n">
         <v>1771354.5</v>
-      </c>
-      <c r="E4" t="n">
-        <v>0</v>
       </c>
       <c r="F4" t="n">
         <v>1771354.5</v>

</xml_diff>